<commit_message>
feat: ping marker delta
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\ElinTogether\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8861D3BA-B051-40C4-9565-53F618C62D32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3476C28-C747-4100-B000-E60801B53074}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4365" yWindow="2250" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11490" yWindow="2685" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="126">
   <si>
     <t>id</t>
   </si>
@@ -397,6 +397,12 @@
   </si>
   <si>
     <t>Elin Together build version mismatch</t>
+  </si>
+  <si>
+    <t>emp_ui_ping</t>
+  </si>
+  <si>
+    <t>{0} pinged a location.</t>
   </si>
 </sst>
 </file>
@@ -736,7 +742,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1432,6 +1438,17 @@
         <v>123</v>
       </c>
     </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>124</v>
+      </c>
+      <c r="C64" t="s">
+        <v>125</v>
+      </c>
+      <c r="D64" t="s">
+        <v>125</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: dialog keymap for ping
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\ElinTogether\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{924746AB-AE14-47C7-A439-17D3BAC7C737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{567A9D0D-0FC8-48C6-B757-55B6FDE52602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11490" yWindow="2685" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="287">
   <si>
     <t>id</t>
   </si>
@@ -774,15 +774,6 @@
   </si>
   <si>
     <t>Kick</t>
-  </si>
-  <si>
-    <t>emp_ui_chat_keymap</t>
-  </si>
-  <si>
-    <t>キー設定: {0}</t>
-  </si>
-  <si>
-    <t>Bind Key: {0}</t>
   </si>
   <si>
     <t>emp_ui_ping_action</t>
@@ -2177,167 +2168,167 @@
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>245</v>
+        <v>185</v>
       </c>
       <c r="C85" t="s">
-        <v>246</v>
+        <v>186</v>
       </c>
       <c r="D85" t="s">
-        <v>247</v>
+        <v>187</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="C86" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D86" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C87" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D87" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C88" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D88" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="C89" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D89" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C90" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D90" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="C91" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D91" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C92" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D92" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="C93" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="D93" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="C94" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D94" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="C95" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="D95" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="C96" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D96" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="C97" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="D97" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="C98" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="D98" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="C99" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D99" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: steam lobby misc changes
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\ElinTogether\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{567A9D0D-0FC8-48C6-B757-55B6FDE52602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{140A520F-4960-4C9C-9607-6C9B0F30C344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11490" yWindow="2685" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="288">
   <si>
     <t>id</t>
   </si>
@@ -442,9 +442,6 @@
   </si>
   <si>
     <t>{0} のゲーム [{1}、{2} 人プレイ、場所: {3}</t>
-  </si>
-  <si>
-    <t>{0}'s Game [{1} with {2} Player, at {3}</t>
   </si>
   <si>
     <t>emp_ui_lobby_tally</t>
@@ -900,6 +897,12 @@
   </si>
   <si>
     <t>All</t>
+  </si>
+  <si>
+    <t>{0}'s Game {1} with {2} Player, at {3}</t>
+  </si>
+  <si>
+    <t>{0} のゲーム  {1}、{2} 人プレイ、場所: {3}</t>
   </si>
 </sst>
 </file>
@@ -1764,125 +1767,125 @@
         <v>137</v>
       </c>
       <c r="C48" t="s">
-        <v>138</v>
+        <v>287</v>
       </c>
       <c r="D48" t="s">
-        <v>139</v>
+        <v>286</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>139</v>
+      </c>
+      <c r="C49" t="s">
         <v>140</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49" t="s">
         <v>141</v>
-      </c>
-      <c r="D49" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>142</v>
+      </c>
+      <c r="C50" t="s">
         <v>143</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>144</v>
-      </c>
-      <c r="D50" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>145</v>
+      </c>
+      <c r="C51" t="s">
         <v>146</v>
       </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
         <v>147</v>
-      </c>
-      <c r="D51" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>148</v>
+      </c>
+      <c r="C52" t="s">
         <v>149</v>
       </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
         <v>150</v>
-      </c>
-      <c r="D52" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>151</v>
+      </c>
+      <c r="C53" t="s">
         <v>152</v>
       </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
         <v>153</v>
-      </c>
-      <c r="D53" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>154</v>
+      </c>
+      <c r="C54" t="s">
         <v>155</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>156</v>
-      </c>
-      <c r="D54" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>157</v>
+      </c>
+      <c r="C55" t="s">
         <v>158</v>
       </c>
-      <c r="C55" t="s">
+      <c r="D55" t="s">
         <v>159</v>
-      </c>
-      <c r="D55" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>160</v>
+      </c>
+      <c r="C56" t="s">
         <v>161</v>
       </c>
-      <c r="C56" t="s">
+      <c r="D56" t="s">
         <v>162</v>
-      </c>
-      <c r="D56" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>163</v>
+      </c>
+      <c r="C57" t="s">
         <v>164</v>
       </c>
-      <c r="C57" t="s">
+      <c r="D57" t="s">
         <v>165</v>
-      </c>
-      <c r="D57" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>166</v>
+      </c>
+      <c r="C58" t="s">
         <v>167</v>
       </c>
-      <c r="C58" t="s">
+      <c r="D58" t="s">
         <v>168</v>
-      </c>
-      <c r="D58" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C59" t="s">
         <v>102</v>
@@ -1893,442 +1896,442 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>170</v>
+      </c>
+      <c r="C60" t="s">
         <v>171</v>
       </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
         <v>172</v>
-      </c>
-      <c r="D60" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>173</v>
+      </c>
+      <c r="C61" t="s">
         <v>174</v>
       </c>
-      <c r="C61" t="s">
-        <v>175</v>
-      </c>
       <c r="D61" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>175</v>
+      </c>
+      <c r="C62" t="s">
         <v>176</v>
       </c>
-      <c r="C62" t="s">
+      <c r="D62" t="s">
         <v>177</v>
-      </c>
-      <c r="D62" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>178</v>
+      </c>
+      <c r="C63" t="s">
         <v>179</v>
       </c>
-      <c r="C63" t="s">
+      <c r="D63" t="s">
         <v>180</v>
-      </c>
-      <c r="D63" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>181</v>
+      </c>
+      <c r="C64" t="s">
         <v>182</v>
       </c>
-      <c r="C64" t="s">
+      <c r="D64" t="s">
         <v>183</v>
-      </c>
-      <c r="D64" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>184</v>
+      </c>
+      <c r="C65" t="s">
         <v>185</v>
       </c>
-      <c r="C65" t="s">
+      <c r="D65" t="s">
         <v>186</v>
-      </c>
-      <c r="D65" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>187</v>
+      </c>
+      <c r="C66" t="s">
         <v>188</v>
       </c>
-      <c r="C66" t="s">
+      <c r="D66" t="s">
         <v>189</v>
-      </c>
-      <c r="D66" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>190</v>
+      </c>
+      <c r="C67" t="s">
         <v>191</v>
       </c>
-      <c r="C67" t="s">
+      <c r="D67" t="s">
         <v>192</v>
-      </c>
-      <c r="D67" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>193</v>
+      </c>
+      <c r="C68" t="s">
         <v>194</v>
       </c>
-      <c r="C68" t="s">
+      <c r="D68" t="s">
         <v>195</v>
-      </c>
-      <c r="D68" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>196</v>
+      </c>
+      <c r="C69" t="s">
         <v>197</v>
       </c>
-      <c r="C69" t="s">
+      <c r="D69" t="s">
         <v>198</v>
-      </c>
-      <c r="D69" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>199</v>
+      </c>
+      <c r="C70" t="s">
         <v>200</v>
       </c>
-      <c r="C70" t="s">
+      <c r="D70" t="s">
         <v>201</v>
-      </c>
-      <c r="D70" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>202</v>
+      </c>
+      <c r="C71" t="s">
         <v>203</v>
       </c>
-      <c r="C71" t="s">
+      <c r="D71" t="s">
         <v>204</v>
-      </c>
-      <c r="D71" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>205</v>
+      </c>
+      <c r="C72" t="s">
         <v>206</v>
       </c>
-      <c r="C72" t="s">
+      <c r="D72" t="s">
         <v>207</v>
-      </c>
-      <c r="D72" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>208</v>
+      </c>
+      <c r="C73" t="s">
         <v>209</v>
       </c>
-      <c r="C73" t="s">
+      <c r="D73" t="s">
         <v>210</v>
-      </c>
-      <c r="D73" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>211</v>
+      </c>
+      <c r="C74" t="s">
         <v>212</v>
       </c>
-      <c r="C74" t="s">
+      <c r="D74" t="s">
         <v>213</v>
-      </c>
-      <c r="D74" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>214</v>
+      </c>
+      <c r="C75" t="s">
         <v>215</v>
       </c>
-      <c r="C75" t="s">
+      <c r="D75" t="s">
         <v>216</v>
-      </c>
-      <c r="D75" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>217</v>
+      </c>
+      <c r="C76" t="s">
         <v>218</v>
       </c>
-      <c r="C76" t="s">
+      <c r="D76" t="s">
         <v>219</v>
-      </c>
-      <c r="D76" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>220</v>
+      </c>
+      <c r="C77" t="s">
         <v>221</v>
       </c>
-      <c r="C77" t="s">
+      <c r="D77" t="s">
         <v>222</v>
-      </c>
-      <c r="D77" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>223</v>
+      </c>
+      <c r="C78" t="s">
         <v>224</v>
       </c>
-      <c r="C78" t="s">
+      <c r="D78" t="s">
         <v>225</v>
-      </c>
-      <c r="D78" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>226</v>
+      </c>
+      <c r="C79" t="s">
         <v>227</v>
       </c>
-      <c r="C79" t="s">
+      <c r="D79" t="s">
         <v>228</v>
-      </c>
-      <c r="D79" t="s">
-        <v>229</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>229</v>
+      </c>
+      <c r="C80" t="s">
         <v>230</v>
       </c>
-      <c r="C80" t="s">
+      <c r="D80" t="s">
         <v>231</v>
-      </c>
-      <c r="D80" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>232</v>
+      </c>
+      <c r="C81" t="s">
         <v>233</v>
       </c>
-      <c r="C81" t="s">
+      <c r="D81" t="s">
         <v>234</v>
-      </c>
-      <c r="D81" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>235</v>
+      </c>
+      <c r="C82" t="s">
         <v>236</v>
       </c>
-      <c r="C82" t="s">
+      <c r="D82" t="s">
         <v>237</v>
-      </c>
-      <c r="D82" t="s">
-        <v>238</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>238</v>
+      </c>
+      <c r="C83" t="s">
         <v>239</v>
       </c>
-      <c r="C83" t="s">
+      <c r="D83" t="s">
         <v>240</v>
-      </c>
-      <c r="D83" t="s">
-        <v>241</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>241</v>
+      </c>
+      <c r="C84" t="s">
         <v>242</v>
       </c>
-      <c r="C84" t="s">
+      <c r="D84" t="s">
         <v>243</v>
-      </c>
-      <c r="D84" t="s">
-        <v>244</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>184</v>
+      </c>
+      <c r="C85" t="s">
         <v>185</v>
       </c>
-      <c r="C85" t="s">
+      <c r="D85" t="s">
         <v>186</v>
-      </c>
-      <c r="D85" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>244</v>
+      </c>
+      <c r="C86" t="s">
         <v>245</v>
       </c>
-      <c r="C86" t="s">
+      <c r="D86" t="s">
         <v>246</v>
-      </c>
-      <c r="D86" t="s">
-        <v>247</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>247</v>
+      </c>
+      <c r="C87" t="s">
         <v>248</v>
       </c>
-      <c r="C87" t="s">
+      <c r="D87" t="s">
         <v>249</v>
-      </c>
-      <c r="D87" t="s">
-        <v>250</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>250</v>
+      </c>
+      <c r="C88" t="s">
         <v>251</v>
       </c>
-      <c r="C88" t="s">
+      <c r="D88" t="s">
         <v>252</v>
-      </c>
-      <c r="D88" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>253</v>
+      </c>
+      <c r="C89" t="s">
         <v>254</v>
       </c>
-      <c r="C89" t="s">
+      <c r="D89" t="s">
         <v>255</v>
-      </c>
-      <c r="D89" t="s">
-        <v>256</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
+        <v>256</v>
+      </c>
+      <c r="C90" t="s">
         <v>257</v>
       </c>
-      <c r="C90" t="s">
+      <c r="D90" t="s">
         <v>258</v>
-      </c>
-      <c r="D90" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
+        <v>259</v>
+      </c>
+      <c r="C91" t="s">
         <v>260</v>
       </c>
-      <c r="C91" t="s">
+      <c r="D91" t="s">
         <v>261</v>
-      </c>
-      <c r="D91" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>262</v>
+      </c>
+      <c r="C92" t="s">
         <v>263</v>
       </c>
-      <c r="C92" t="s">
+      <c r="D92" t="s">
         <v>264</v>
-      </c>
-      <c r="D92" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>265</v>
+      </c>
+      <c r="C93" t="s">
         <v>266</v>
       </c>
-      <c r="C93" t="s">
+      <c r="D93" t="s">
         <v>267</v>
-      </c>
-      <c r="D93" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
+        <v>268</v>
+      </c>
+      <c r="C94" t="s">
         <v>269</v>
       </c>
-      <c r="C94" t="s">
+      <c r="D94" t="s">
         <v>270</v>
-      </c>
-      <c r="D94" t="s">
-        <v>271</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
+        <v>271</v>
+      </c>
+      <c r="C95" t="s">
         <v>272</v>
       </c>
-      <c r="C95" t="s">
+      <c r="D95" t="s">
         <v>273</v>
-      </c>
-      <c r="D95" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>274</v>
+      </c>
+      <c r="C96" t="s">
         <v>275</v>
       </c>
-      <c r="C96" t="s">
+      <c r="D96" t="s">
         <v>276</v>
-      </c>
-      <c r="D96" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
+        <v>277</v>
+      </c>
+      <c r="C97" t="s">
         <v>278</v>
       </c>
-      <c r="C97" t="s">
+      <c r="D97" t="s">
         <v>279</v>
-      </c>
-      <c r="D97" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>280</v>
+      </c>
+      <c r="C98" t="s">
         <v>281</v>
       </c>
-      <c r="C98" t="s">
+      <c r="D98" t="s">
         <v>282</v>
-      </c>
-      <c r="D98" t="s">
-        <v>283</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
+        <v>283</v>
+      </c>
+      <c r="C99" t="s">
         <v>284</v>
       </c>
-      <c r="C99" t="s">
+      <c r="D99" t="s">
         <v>285</v>
-      </c>
-      <c r="D99" t="s">
-        <v>286</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: host force reconnect & session sync request
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\ElinTogether\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{140A520F-4960-4C9C-9607-6C9B0F30C344}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4374541-DF47-4FF9-AB3F-A6EBDB686FE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11490" yWindow="2685" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11940" yWindow="2565" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="292">
   <si>
     <t>id</t>
   </si>
@@ -439,9 +439,6 @@
   </si>
   <si>
     <t>emp_ui_lobby_desc</t>
-  </si>
-  <si>
-    <t>{0} のゲーム [{1}、{2} 人プレイ、場所: {3}</t>
   </si>
   <si>
     <t>emp_ui_lobby_tally</t>
@@ -903,6 +900,21 @@
   </si>
   <si>
     <t>{0} のゲーム  {1}、{2} 人プレイ、場所: {3}</t>
+  </si>
+  <si>
+    <t>emp_ui_reconnect</t>
+  </si>
+  <si>
+    <t>Reconnect</t>
+  </si>
+  <si>
+    <t>再接続</t>
+  </si>
+  <si>
+    <t>emp_dc_reconnect_request</t>
+  </si>
+  <si>
+    <t>Reconnect Request</t>
   </si>
 </sst>
 </file>
@@ -1242,7 +1254,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D99"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1767,125 +1779,125 @@
         <v>137</v>
       </c>
       <c r="C48" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D48" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>138</v>
+      </c>
+      <c r="C49" t="s">
         <v>139</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49" t="s">
         <v>140</v>
-      </c>
-      <c r="D49" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
+        <v>141</v>
+      </c>
+      <c r="C50" t="s">
         <v>142</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>143</v>
-      </c>
-      <c r="D50" t="s">
-        <v>144</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
+        <v>144</v>
+      </c>
+      <c r="C51" t="s">
         <v>145</v>
       </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
         <v>146</v>
-      </c>
-      <c r="D51" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
+        <v>147</v>
+      </c>
+      <c r="C52" t="s">
         <v>148</v>
       </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
         <v>149</v>
-      </c>
-      <c r="D52" t="s">
-        <v>150</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
+        <v>150</v>
+      </c>
+      <c r="C53" t="s">
         <v>151</v>
       </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
         <v>152</v>
-      </c>
-      <c r="D53" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
+        <v>153</v>
+      </c>
+      <c r="C54" t="s">
         <v>154</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>155</v>
-      </c>
-      <c r="D54" t="s">
-        <v>156</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
+        <v>156</v>
+      </c>
+      <c r="C55" t="s">
         <v>157</v>
       </c>
-      <c r="C55" t="s">
+      <c r="D55" t="s">
         <v>158</v>
-      </c>
-      <c r="D55" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
+        <v>159</v>
+      </c>
+      <c r="C56" t="s">
         <v>160</v>
       </c>
-      <c r="C56" t="s">
+      <c r="D56" t="s">
         <v>161</v>
-      </c>
-      <c r="D56" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
+        <v>162</v>
+      </c>
+      <c r="C57" t="s">
         <v>163</v>
       </c>
-      <c r="C57" t="s">
+      <c r="D57" t="s">
         <v>164</v>
-      </c>
-      <c r="D57" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
+        <v>165</v>
+      </c>
+      <c r="C58" t="s">
         <v>166</v>
       </c>
-      <c r="C58" t="s">
+      <c r="D58" t="s">
         <v>167</v>
-      </c>
-      <c r="D58" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C59" t="s">
         <v>102</v>
@@ -1896,442 +1908,464 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>169</v>
+      </c>
+      <c r="C60" t="s">
         <v>170</v>
       </c>
-      <c r="C60" t="s">
+      <c r="D60" t="s">
         <v>171</v>
-      </c>
-      <c r="D60" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
+        <v>172</v>
+      </c>
+      <c r="C61" t="s">
         <v>173</v>
       </c>
-      <c r="C61" t="s">
-        <v>174</v>
-      </c>
       <c r="D61" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
+        <v>174</v>
+      </c>
+      <c r="C62" t="s">
         <v>175</v>
       </c>
-      <c r="C62" t="s">
+      <c r="D62" t="s">
         <v>176</v>
-      </c>
-      <c r="D62" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>177</v>
+      </c>
+      <c r="C63" t="s">
         <v>178</v>
       </c>
-      <c r="C63" t="s">
+      <c r="D63" t="s">
         <v>179</v>
-      </c>
-      <c r="D63" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>180</v>
+      </c>
+      <c r="C64" t="s">
         <v>181</v>
       </c>
-      <c r="C64" t="s">
+      <c r="D64" t="s">
         <v>182</v>
-      </c>
-      <c r="D64" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>183</v>
+      </c>
+      <c r="C65" t="s">
         <v>184</v>
       </c>
-      <c r="C65" t="s">
+      <c r="D65" t="s">
         <v>185</v>
-      </c>
-      <c r="D65" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>186</v>
+      </c>
+      <c r="C66" t="s">
         <v>187</v>
       </c>
-      <c r="C66" t="s">
+      <c r="D66" t="s">
         <v>188</v>
-      </c>
-      <c r="D66" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>189</v>
+      </c>
+      <c r="C67" t="s">
         <v>190</v>
       </c>
-      <c r="C67" t="s">
+      <c r="D67" t="s">
         <v>191</v>
-      </c>
-      <c r="D67" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>192</v>
+      </c>
+      <c r="C68" t="s">
         <v>193</v>
       </c>
-      <c r="C68" t="s">
+      <c r="D68" t="s">
         <v>194</v>
-      </c>
-      <c r="D68" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>195</v>
+      </c>
+      <c r="C69" t="s">
         <v>196</v>
       </c>
-      <c r="C69" t="s">
+      <c r="D69" t="s">
         <v>197</v>
-      </c>
-      <c r="D69" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>198</v>
+      </c>
+      <c r="C70" t="s">
         <v>199</v>
       </c>
-      <c r="C70" t="s">
+      <c r="D70" t="s">
         <v>200</v>
-      </c>
-      <c r="D70" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
+        <v>201</v>
+      </c>
+      <c r="C71" t="s">
         <v>202</v>
       </c>
-      <c r="C71" t="s">
+      <c r="D71" t="s">
         <v>203</v>
-      </c>
-      <c r="D71" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
+        <v>204</v>
+      </c>
+      <c r="C72" t="s">
         <v>205</v>
       </c>
-      <c r="C72" t="s">
+      <c r="D72" t="s">
         <v>206</v>
-      </c>
-      <c r="D72" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
+        <v>207</v>
+      </c>
+      <c r="C73" t="s">
         <v>208</v>
       </c>
-      <c r="C73" t="s">
+      <c r="D73" t="s">
         <v>209</v>
-      </c>
-      <c r="D73" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
+        <v>210</v>
+      </c>
+      <c r="C74" t="s">
         <v>211</v>
       </c>
-      <c r="C74" t="s">
+      <c r="D74" t="s">
         <v>212</v>
-      </c>
-      <c r="D74" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>213</v>
+      </c>
+      <c r="C75" t="s">
         <v>214</v>
       </c>
-      <c r="C75" t="s">
+      <c r="D75" t="s">
         <v>215</v>
-      </c>
-      <c r="D75" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>216</v>
+      </c>
+      <c r="C76" t="s">
         <v>217</v>
       </c>
-      <c r="C76" t="s">
+      <c r="D76" t="s">
         <v>218</v>
-      </c>
-      <c r="D76" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>219</v>
+      </c>
+      <c r="C77" t="s">
         <v>220</v>
       </c>
-      <c r="C77" t="s">
+      <c r="D77" t="s">
         <v>221</v>
-      </c>
-      <c r="D77" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>222</v>
+      </c>
+      <c r="C78" t="s">
         <v>223</v>
       </c>
-      <c r="C78" t="s">
+      <c r="D78" t="s">
         <v>224</v>
-      </c>
-      <c r="D78" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>225</v>
+      </c>
+      <c r="C79" t="s">
         <v>226</v>
       </c>
-      <c r="C79" t="s">
+      <c r="D79" t="s">
         <v>227</v>
-      </c>
-      <c r="D79" t="s">
-        <v>228</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>228</v>
+      </c>
+      <c r="C80" t="s">
         <v>229</v>
       </c>
-      <c r="C80" t="s">
+      <c r="D80" t="s">
         <v>230</v>
-      </c>
-      <c r="D80" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>231</v>
+      </c>
+      <c r="C81" t="s">
         <v>232</v>
       </c>
-      <c r="C81" t="s">
+      <c r="D81" t="s">
         <v>233</v>
-      </c>
-      <c r="D81" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>234</v>
+      </c>
+      <c r="C82" t="s">
         <v>235</v>
       </c>
-      <c r="C82" t="s">
+      <c r="D82" t="s">
         <v>236</v>
-      </c>
-      <c r="D82" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
+        <v>237</v>
+      </c>
+      <c r="C83" t="s">
         <v>238</v>
       </c>
-      <c r="C83" t="s">
+      <c r="D83" t="s">
         <v>239</v>
-      </c>
-      <c r="D83" t="s">
-        <v>240</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
+        <v>240</v>
+      </c>
+      <c r="C84" t="s">
         <v>241</v>
       </c>
-      <c r="C84" t="s">
+      <c r="D84" t="s">
         <v>242</v>
-      </c>
-      <c r="D84" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
+        <v>183</v>
+      </c>
+      <c r="C85" t="s">
         <v>184</v>
       </c>
-      <c r="C85" t="s">
+      <c r="D85" t="s">
         <v>185</v>
-      </c>
-      <c r="D85" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
+        <v>243</v>
+      </c>
+      <c r="C86" t="s">
         <v>244</v>
       </c>
-      <c r="C86" t="s">
+      <c r="D86" t="s">
         <v>245</v>
-      </c>
-      <c r="D86" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
+        <v>246</v>
+      </c>
+      <c r="C87" t="s">
         <v>247</v>
       </c>
-      <c r="C87" t="s">
+      <c r="D87" t="s">
         <v>248</v>
-      </c>
-      <c r="D87" t="s">
-        <v>249</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
+        <v>249</v>
+      </c>
+      <c r="C88" t="s">
         <v>250</v>
       </c>
-      <c r="C88" t="s">
+      <c r="D88" t="s">
         <v>251</v>
-      </c>
-      <c r="D88" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
+        <v>252</v>
+      </c>
+      <c r="C89" t="s">
         <v>253</v>
       </c>
-      <c r="C89" t="s">
+      <c r="D89" t="s">
         <v>254</v>
-      </c>
-      <c r="D89" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
+        <v>255</v>
+      </c>
+      <c r="C90" t="s">
         <v>256</v>
       </c>
-      <c r="C90" t="s">
+      <c r="D90" t="s">
         <v>257</v>
-      </c>
-      <c r="D90" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
+        <v>258</v>
+      </c>
+      <c r="C91" t="s">
         <v>259</v>
       </c>
-      <c r="C91" t="s">
+      <c r="D91" t="s">
         <v>260</v>
-      </c>
-      <c r="D91" t="s">
-        <v>261</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
+        <v>261</v>
+      </c>
+      <c r="C92" t="s">
         <v>262</v>
       </c>
-      <c r="C92" t="s">
+      <c r="D92" t="s">
         <v>263</v>
-      </c>
-      <c r="D92" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
+        <v>264</v>
+      </c>
+      <c r="C93" t="s">
         <v>265</v>
       </c>
-      <c r="C93" t="s">
+      <c r="D93" t="s">
         <v>266</v>
-      </c>
-      <c r="D93" t="s">
-        <v>267</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
+        <v>267</v>
+      </c>
+      <c r="C94" t="s">
         <v>268</v>
       </c>
-      <c r="C94" t="s">
+      <c r="D94" t="s">
         <v>269</v>
-      </c>
-      <c r="D94" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
+        <v>270</v>
+      </c>
+      <c r="C95" t="s">
         <v>271</v>
       </c>
-      <c r="C95" t="s">
+      <c r="D95" t="s">
         <v>272</v>
-      </c>
-      <c r="D95" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>273</v>
+      </c>
+      <c r="C96" t="s">
         <v>274</v>
       </c>
-      <c r="C96" t="s">
+      <c r="D96" t="s">
         <v>275</v>
-      </c>
-      <c r="D96" t="s">
-        <v>276</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
+        <v>276</v>
+      </c>
+      <c r="C97" t="s">
         <v>277</v>
       </c>
-      <c r="C97" t="s">
+      <c r="D97" t="s">
         <v>278</v>
-      </c>
-      <c r="D97" t="s">
-        <v>279</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>279</v>
+      </c>
+      <c r="C98" t="s">
         <v>280</v>
       </c>
-      <c r="C98" t="s">
+      <c r="D98" t="s">
         <v>281</v>
-      </c>
-      <c r="D98" t="s">
-        <v>282</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
+        <v>282</v>
+      </c>
+      <c r="C99" t="s">
         <v>283</v>
       </c>
-      <c r="C99" t="s">
+      <c r="D99" t="s">
         <v>284</v>
       </c>
-      <c r="D99" t="s">
-        <v>285</v>
+    </row>
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>287</v>
+      </c>
+      <c r="C100" t="s">
+        <v>289</v>
+      </c>
+      <c r="D100" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>290</v>
+      </c>
+      <c r="C101" t="s">
+        <v>289</v>
+      </c>
+      <c r="D101" t="s">
+        <v>291</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: lobby reconnect & ui cleanups
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\ElinTogether\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26C74E31-E182-4F2A-8517-DFA94FC3089A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F1CAB91-18DC-4A34-9D67-54A049E401FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11940" yWindow="2565" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11505" yWindow="1980" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="301">
   <si>
     <t>id</t>
   </si>
@@ -869,18 +869,12 @@
     <t>None</t>
   </si>
   <si>
-    <t>emp_validation_source</t>
-  </si>
-  <si>
     <t>ソース</t>
   </si>
   <si>
     <t>Source</t>
   </si>
   <si>
-    <t>emp_validation_plugin</t>
-  </si>
-  <si>
     <t>プラグイン</t>
   </si>
   <si>
@@ -915,6 +909,41 @@
   </si>
   <si>
     <t>Reconnect Request</t>
+  </si>
+  <si>
+    <t>emp_lobby_create_failed</t>
+  </si>
+  <si>
+    <t>emp_lobby_enter_failed</t>
+  </si>
+  <si>
+    <t>emp_lobby_already_joined</t>
+  </si>
+  <si>
+    <t>Failed to create Steam lobby: {Result}
+Try again later</t>
+  </si>
+  <si>
+    <t>Failed to enter Steam lobby: {Response}</t>
+  </si>
+  <si>
+    <t>Already in the same lobby</t>
+  </si>
+  <si>
+    <t>Steamロビーへの参加に失敗しました: {Response}</t>
+  </si>
+  <si>
+    <t>すでに同じロビーに参加しています</t>
+  </si>
+  <si>
+    <t>Steamロビーの作成に失敗しました: {Result}
+後でもう一度試してください</t>
+  </si>
+  <si>
+    <t>emp_validation_sources</t>
+  </si>
+  <si>
+    <t>emp_validation_plugins</t>
   </si>
 </sst>
 </file>
@@ -950,8 +979,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1254,7 +1286,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:D104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1779,10 +1811,10 @@
         <v>137</v>
       </c>
       <c r="C48" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="D48" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -2126,14 +2158,14 @@
         <v>227</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" ht="60" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>228</v>
       </c>
       <c r="C80" t="s">
         <v>229</v>
       </c>
-      <c r="D80" t="s">
+      <c r="D80" s="1" t="s">
         <v>230</v>
       </c>
     </row>
@@ -2315,57 +2347,90 @@
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
+        <v>299</v>
+      </c>
+      <c r="C97" t="s">
         <v>276</v>
       </c>
-      <c r="C97" t="s">
+      <c r="D97" t="s">
         <v>277</v>
-      </c>
-      <c r="D97" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>300</v>
+      </c>
+      <c r="C98" t="s">
+        <v>278</v>
+      </c>
+      <c r="D98" t="s">
         <v>279</v>
-      </c>
-      <c r="C98" t="s">
-        <v>280</v>
-      </c>
-      <c r="D98" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
+        <v>280</v>
+      </c>
+      <c r="C99" t="s">
+        <v>281</v>
+      </c>
+      <c r="D99" t="s">
         <v>282</v>
-      </c>
-      <c r="C99" t="s">
-        <v>283</v>
-      </c>
-      <c r="D99" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
+        <v>285</v>
+      </c>
+      <c r="C100" t="s">
         <v>287</v>
       </c>
-      <c r="C100" t="s">
-        <v>289</v>
-      </c>
       <c r="D100" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
+        <v>288</v>
+      </c>
+      <c r="C101" t="s">
+        <v>287</v>
+      </c>
+      <c r="D101" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
         <v>290</v>
       </c>
-      <c r="C101" t="s">
-        <v>289</v>
-      </c>
-      <c r="D101" t="s">
+      <c r="C102" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
         <v>291</v>
+      </c>
+      <c r="C103" t="s">
+        <v>296</v>
+      </c>
+      <c r="D103" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>292</v>
+      </c>
+      <c r="C104" t="s">
+        <v>297</v>
+      </c>
+      <c r="D104" t="s">
+        <v>295</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(temp): disable client click quest
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\ElinTogether\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F1CAB91-18DC-4A34-9D67-54A049E401FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6630F41-19DB-4A7B-B15E-FAA06CAEE813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11505" yWindow="1980" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="311" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="304">
   <si>
     <t>id</t>
   </si>
@@ -944,6 +944,15 @@
   </si>
   <si>
     <t>emp_validation_plugins</t>
+  </si>
+  <si>
+    <t>emp_ui_quest_client</t>
+  </si>
+  <si>
+    <t>(Temp) Clients can't accept quests</t>
+  </si>
+  <si>
+    <t>（暫定）クライアントがクエストを受諾できない</t>
   </si>
 </sst>
 </file>
@@ -1286,7 +1295,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D104"/>
+  <dimension ref="A1:D105"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -2433,6 +2442,17 @@
         <v>295</v>
       </c>
     </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>301</v>
+      </c>
+      <c r="C105" t="s">
+        <v>303</v>
+      </c>
+      <c r="D105" t="s">
+        <v>302</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: partial client quest sync
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\ElinTogether\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6630F41-19DB-4A7B-B15E-FAA06CAEE813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B230DB-B1A1-4D4B-8AE1-023DE6B04A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11505" yWindow="1980" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -949,10 +949,10 @@
     <t>emp_ui_quest_client</t>
   </si>
   <si>
-    <t>(Temp) Clients can't accept quests</t>
-  </si>
-  <si>
-    <t>（暫定）クライアントがクエストを受諾できない</t>
+    <t>(Temp) This quest cannot be started by client players.</t>
+  </si>
+  <si>
+    <t>（暫定）このクエストはクライアントプレイヤーからは開始できません。</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
feat: enchance build version integrity check
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\ElinTogether\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07B230DB-B1A1-4D4B-8AE1-023DE6B04A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF11724-B9B8-43EC-B9B0-AFD3A16D3695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11505" yWindow="1980" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22635" yWindow="2130" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="314" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="319">
   <si>
     <t>id</t>
   </si>
@@ -797,15 +797,6 @@
     <t>Source validation failed — {0} mismatches</t>
   </si>
   <si>
-    <t>emp_ui_source_mismatch_acts</t>
-  </si>
-  <si>
-    <t>Act 不一致:</t>
-  </si>
-  <si>
-    <t>Act mismatches:</t>
-  </si>
-  <si>
     <t>emp_ui_source_mismatch_sources</t>
   </si>
   <si>
@@ -953,6 +944,74 @@
   </si>
   <si>
     <t>（暫定）このクエストはクライアントプレイヤーからは開始できません。</t>
+  </si>
+  <si>
+    <t>emp_dc_version_mismatch</t>
+  </si>
+  <si>
+    <t>emp_dc_act_mismatch</t>
+  </si>
+  <si>
+    <t>Disconnected: invalid version</t>
+  </si>
+  <si>
+    <t>切断: 無効なVersion</t>
+  </si>
+  <si>
+    <t>切断: Act 不一致</t>
+  </si>
+  <si>
+    <t>Act mapping mismatch</t>
+  </si>
+  <si>
+    <t>emp_ui_reject_acts</t>
+  </si>
+  <si>
+    <t>emp_ui_reject_integrity</t>
+  </si>
+  <si>
+    <t>emp_version_rejected_host</t>
+  </si>
+  <si>
+    <t>emp_version_rejected_client</t>
+  </si>
+  <si>
+    <t>Could not join: Host has strict verification enabled. Data integrity mismatch ({0})</t>
+  </si>
+  <si>
+    <t>Could not join: Act mapping mismatch ({0})
+Act ID is used for action sync. Game cannot run with mismatch acts.
+Please ensure both players have the exact same mods installed.</t>
+  </si>
+  <si>
+    <t>Connection request from {0} rejected
+Version mismatch with host
+Host Mod: {1}
+Host Game: {2}</t>
+  </si>
+  <si>
+    <t>Could not join: Version mismatch
+Mod: Local {0} / Host {1}
+Game: Local {2} / Host {3}</t>
+  </si>
+  <si>
+    <t>参加できません：Actマッピングが一致しません（{0}件）
+Act ID同期エラー：不一致は動作不良の原因になります。
+双方とも同じModを導入しているか確認してください。</t>
+  </si>
+  <si>
+    <t>参加できません：ホストの厳密チェックにより、データ整合性が不一致です（{0}件）</t>
+  </si>
+  <si>
+    <t>{0}の接続を拒否しました
+バージョンがホストと一致しません
+ホストMod：{1}
+ホストゲーム：{2}</t>
+  </si>
+  <si>
+    <t>参加できません：バージョン不一致
+Mod：自機 {0} ／ ホスト {1}
+ゲーム：自機 {2} ／ ホスト {3}</t>
   </si>
 </sst>
 </file>
@@ -1295,7 +1354,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D105"/>
+  <dimension ref="A1:D110"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1820,10 +1879,10 @@
         <v>137</v>
       </c>
       <c r="C48" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="D48" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
@@ -2345,29 +2404,29 @@
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
+        <v>296</v>
+      </c>
+      <c r="C96" t="s">
         <v>273</v>
       </c>
-      <c r="C96" t="s">
+      <c r="D96" t="s">
         <v>274</v>
-      </c>
-      <c r="D96" t="s">
-        <v>275</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C97" t="s">
+        <v>275</v>
+      </c>
+      <c r="D97" t="s">
         <v>276</v>
-      </c>
-      <c r="D97" t="s">
-        <v>277</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>300</v>
+        <v>277</v>
       </c>
       <c r="C98" t="s">
         <v>278</v>
@@ -2378,13 +2437,13 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C99" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="D99" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
@@ -2392,54 +2451,54 @@
         <v>285</v>
       </c>
       <c r="C100" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="D100" t="s">
         <v>286</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
+        <v>287</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
         <v>288</v>
       </c>
-      <c r="C101" t="s">
-        <v>287</v>
-      </c>
-      <c r="D101" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="102" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A102" t="s">
-        <v>290</v>
-      </c>
-      <c r="C102" s="1" t="s">
-        <v>298</v>
-      </c>
-      <c r="D102" s="1" t="s">
+      <c r="C102" t="s">
         <v>293</v>
+      </c>
+      <c r="D102" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C103" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="D103" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="C104" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="D104" t="s">
-        <v>295</v>
+        <v>299</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -2447,10 +2506,65 @@
         <v>301</v>
       </c>
       <c r="C105" t="s">
+        <v>304</v>
+      </c>
+      <c r="D105" t="s">
         <v>303</v>
       </c>
-      <c r="D105" t="s">
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
         <v>302</v>
+      </c>
+      <c r="C106" t="s">
+        <v>305</v>
+      </c>
+      <c r="D106" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>307</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="D107" s="1" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>308</v>
+      </c>
+      <c r="C108" t="s">
+        <v>316</v>
+      </c>
+      <c r="D108" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>309</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>310</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="D110" s="1" t="s">
+        <v>314</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: sleep vote sync
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/emp_localization.xlsx
+++ b/package/LangMod/EN/emp_localization.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WorkSpace\GameMods\ElinTogether\package\LangMod\EN\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF11724-B9B8-43EC-B9B0-AFD3A16D3695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4502DF6-8CDB-413A-8F87-1E3A94E14084}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22635" yWindow="2130" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="2685" windowWidth="31695" windowHeight="18195" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="General" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="328">
   <si>
     <t>id</t>
   </si>
@@ -439,6 +439,12 @@
   </si>
   <si>
     <t>emp_ui_lobby_desc</t>
+  </si>
+  <si>
+    <t>{0} のゲーム  {1}、{2} 人プレイ、場所: {3}</t>
+  </si>
+  <si>
+    <t>{0}'s Game {1} with {2} Player, at {3}</t>
   </si>
   <si>
     <t>emp_ui_lobby_tally</t>
@@ -860,12 +866,18 @@
     <t>None</t>
   </si>
   <si>
+    <t>emp_validation_sources</t>
+  </si>
+  <si>
     <t>ソース</t>
   </si>
   <si>
     <t>Source</t>
   </si>
   <si>
+    <t>emp_validation_plugins</t>
+  </si>
+  <si>
     <t>プラグイン</t>
   </si>
   <si>
@@ -881,21 +893,15 @@
     <t>All</t>
   </si>
   <si>
-    <t>{0}'s Game {1} with {2} Player, at {3}</t>
-  </si>
-  <si>
-    <t>{0} のゲーム  {1}、{2} 人プレイ、場所: {3}</t>
-  </si>
-  <si>
     <t>emp_ui_reconnect</t>
   </si>
   <si>
+    <t>再接続</t>
+  </si>
+  <si>
     <t>Reconnect</t>
   </si>
   <si>
-    <t>再接続</t>
-  </si>
-  <si>
     <t>emp_dc_reconnect_request</t>
   </si>
   <si>
@@ -905,59 +911,53 @@
     <t>emp_lobby_create_failed</t>
   </si>
   <si>
-    <t>emp_lobby_enter_failed</t>
-  </si>
-  <si>
-    <t>emp_lobby_already_joined</t>
+    <t>Steamロビーの作成に失敗しました: {Result}
+後でもう一度試してください</t>
   </si>
   <si>
     <t>Failed to create Steam lobby: {Result}
 Try again later</t>
   </si>
   <si>
+    <t>emp_lobby_enter_failed</t>
+  </si>
+  <si>
+    <t>Steamロビーへの参加に失敗しました: {Response}</t>
+  </si>
+  <si>
     <t>Failed to enter Steam lobby: {Response}</t>
   </si>
   <si>
+    <t>emp_lobby_already_joined</t>
+  </si>
+  <si>
+    <t>すでに同じロビーに参加しています</t>
+  </si>
+  <si>
     <t>Already in the same lobby</t>
   </si>
   <si>
-    <t>Steamロビーへの参加に失敗しました: {Response}</t>
-  </si>
-  <si>
-    <t>すでに同じロビーに参加しています</t>
-  </si>
-  <si>
-    <t>Steamロビーの作成に失敗しました: {Result}
-後でもう一度試してください</t>
-  </si>
-  <si>
-    <t>emp_validation_sources</t>
-  </si>
-  <si>
-    <t>emp_validation_plugins</t>
-  </si>
-  <si>
     <t>emp_ui_quest_client</t>
   </si>
   <si>
+    <t>（暫定）このクエストはクライアントプレイヤーからは開始できません。</t>
+  </si>
+  <si>
     <t>(Temp) This quest cannot be started by client players.</t>
   </si>
   <si>
-    <t>（暫定）このクエストはクライアントプレイヤーからは開始できません。</t>
-  </si>
-  <si>
     <t>emp_dc_version_mismatch</t>
   </si>
   <si>
+    <t>切断: 無効なVersion</t>
+  </si>
+  <si>
+    <t>Disconnected: invalid version</t>
+  </si>
+  <si>
     <t>emp_dc_act_mismatch</t>
   </si>
   <si>
-    <t>Disconnected: invalid version</t>
-  </si>
-  <si>
-    <t>切断: 無効なVersion</t>
-  </si>
-  <si>
     <t>切断: Act 不一致</t>
   </si>
   <si>
@@ -967,21 +967,32 @@
     <t>emp_ui_reject_acts</t>
   </si>
   <si>
-    <t>emp_ui_reject_integrity</t>
-  </si>
-  <si>
-    <t>emp_version_rejected_host</t>
-  </si>
-  <si>
-    <t>emp_version_rejected_client</t>
-  </si>
-  <si>
-    <t>Could not join: Host has strict verification enabled. Data integrity mismatch ({0})</t>
+    <t>参加できません：Actマッピングが一致しません（{0}件）
+Act ID同期エラー：不一致は動作不良の原因になります。
+双方とも同じModを導入しているか確認してください。</t>
   </si>
   <si>
     <t>Could not join: Act mapping mismatch ({0})
 Act ID is used for action sync. Game cannot run with mismatch acts.
 Please ensure both players have the exact same mods installed.</t>
+  </si>
+  <si>
+    <t>emp_ui_reject_integrity</t>
+  </si>
+  <si>
+    <t>参加できません：ホストの厳密チェックにより、データ整合性が不一致です（{0}件）</t>
+  </si>
+  <si>
+    <t>Could not join: Host has strict verification enabled. Data integrity mismatch ({0})</t>
+  </si>
+  <si>
+    <t>emp_version_rejected_host</t>
+  </si>
+  <si>
+    <t>{0}の接続を拒否しました
+バージョンがホストと一致しません
+ホストMod：{1}
+ホストゲーム：{2}</t>
   </si>
   <si>
     <t>Connection request from {0} rejected
@@ -990,28 +1001,44 @@
 Host Game: {2}</t>
   </si>
   <si>
+    <t>emp_version_rejected_client</t>
+  </si>
+  <si>
+    <t>参加できません：バージョン不一致
+Mod：自機 {0} ／ ホスト {1}
+ゲーム：自機 {2} ／ ホスト {3}</t>
+  </si>
+  <si>
     <t>Could not join: Version mismatch
 Mod: Local {0} / Host {1}
 Game: Local {2} / Host {3}</t>
   </si>
   <si>
-    <t>参加できません：Actマッピングが一致しません（{0}件）
-Act ID同期エラー：不一致は動作不良の原因になります。
-双方とも同じModを導入しているか確認してください。</t>
-  </si>
-  <si>
-    <t>参加できません：ホストの厳密チェックにより、データ整合性が不一致です（{0}件）</t>
-  </si>
-  <si>
-    <t>{0}の接続を拒否しました
-バージョンがホストと一致しません
-ホストMod：{1}
-ホストゲーム：{2}</t>
-  </si>
-  <si>
-    <t>参加できません：バージョン不一致
-Mod：自機 {0} ／ ホスト {1}
-ゲーム：自機 {2} ／ ホスト {3}</t>
+    <t>emp_ui_sleep_request</t>
+  </si>
+  <si>
+    <t>emp_ui_sleep_wish</t>
+  </si>
+  <si>
+    <t>{0}が眠りたがっています（{1}/{2}）</t>
+  </si>
+  <si>
+    <t>{0} wants to sleep ({1}/{2})</t>
+  </si>
+  <si>
+    <t>emp_ui_sleep_cancel</t>
+  </si>
+  <si>
+    <t>{0}が目を覚ましました（{1}/{2}）</t>
+  </si>
+  <si>
+    <t>{0} woke up ({1}/{2})</t>
+  </si>
+  <si>
+    <t>Waiting for everyone to go to bed...</t>
+  </si>
+  <si>
+    <t>全員がベッドに入るのを待っています…</t>
   </si>
 </sst>
 </file>
@@ -1354,7 +1381,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D110"/>
+  <dimension ref="A1:D113"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -1879,125 +1906,125 @@
         <v>137</v>
       </c>
       <c r="C48" t="s">
-        <v>281</v>
+        <v>138</v>
       </c>
       <c r="D48" t="s">
-        <v>280</v>
+        <v>139</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C49" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D49" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C50" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D50" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C51" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D51" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C52" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D52" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C53" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D53" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C54" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D54" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C55" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D55" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C56" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D56" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C57" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D57" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C58" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D58" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C59" t="s">
         <v>102</v>
@@ -2008,486 +2035,486 @@
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C60" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D60" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C61" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D61" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C62" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D62" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C63" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D63" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C64" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="D64" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C65" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D65" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C66" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D66" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C67" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D67" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C68" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D68" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C69" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D69" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C70" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D70" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C71" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D71" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C72" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D72" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C73" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D73" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C74" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D74" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="C75" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D75" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C76" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D76" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C77" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D77" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C78" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D78" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C79" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D79" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C80" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C81" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D81" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C82" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D82" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C83" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D83" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C84" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D84" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="C85" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D85" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C86" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D86" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C87" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D87" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C88" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D88" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C89" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="D89" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C90" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D90" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C91" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D91" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C92" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D92" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C93" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="D93" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="C94" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="D94" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C95" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D95" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>296</v>
+        <v>275</v>
       </c>
       <c r="C96" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="D96" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>297</v>
+        <v>278</v>
       </c>
       <c r="C97" t="s">
-        <v>275</v>
+        <v>279</v>
       </c>
       <c r="D97" t="s">
-        <v>276</v>
+        <v>280</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="C98" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="D98" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C99" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D99" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
+        <v>287</v>
+      </c>
+      <c r="C100" t="s">
         <v>285</v>
       </c>
-      <c r="C100" t="s">
-        <v>284</v>
-      </c>
       <c r="D100" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>288</v>
+        <v>292</v>
       </c>
       <c r="C102" t="s">
         <v>293</v>
       </c>
       <c r="D102" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="C103" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D103" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.25">
@@ -2495,10 +2522,10 @@
         <v>298</v>
       </c>
       <c r="C104" t="s">
+        <v>299</v>
+      </c>
+      <c r="D104" t="s">
         <v>300</v>
-      </c>
-      <c r="D104" t="s">
-        <v>299</v>
       </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.25">
@@ -2506,7 +2533,7 @@
         <v>301</v>
       </c>
       <c r="C105" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="D105" t="s">
         <v>303</v>
@@ -2514,7 +2541,7 @@
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C106" t="s">
         <v>305</v>
@@ -2523,48 +2550,81 @@
         <v>306</v>
       </c>
     </row>
-    <row r="107" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>307</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>315</v>
+        <v>308</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="C108" t="s">
+        <v>311</v>
+      </c>
+      <c r="D108" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>313</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="D109" s="1" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
         <v>316</v>
       </c>
-      <c r="D108" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="109" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A109" t="s">
-        <v>309</v>
-      </c>
-      <c r="C109" s="1" t="s">
+      <c r="C110" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="D109" s="1" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="110" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A110" t="s">
-        <v>310</v>
-      </c>
-      <c r="C110" s="1" t="s">
+      <c r="D110" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="D110" s="1" t="s">
-        <v>314</v>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>319</v>
+      </c>
+      <c r="C111" t="s">
+        <v>327</v>
+      </c>
+      <c r="D111" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>320</v>
+      </c>
+      <c r="C112" t="s">
+        <v>321</v>
+      </c>
+      <c r="D112" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>323</v>
+      </c>
+      <c r="C113" t="s">
+        <v>324</v>
+      </c>
+      <c r="D113" t="s">
+        <v>325</v>
       </c>
     </row>
   </sheetData>

</xml_diff>